<commit_message>
Kullanim defteri bos satir kok nedeni: bot.py script olarak calisinca modul adi __main__ oluyor; kaydet'in 'import bot'u IKINCI modul kopyasi yaratip bos sozluk okuyordu (dunku derin satiri dolu, bugunku gunluk bos — bunu kanitliyor). Kaydet artik __main__'deki dolu sozlugue esneği varsa onu okur. Ayrica zincirdeki 3 dogrudan cagri noktasi (ZAI yedek, derin GLM, makro GLM) de _LLM_SON_BASARI'ya kaydediyor. Bugunku bos gunluk satiri log iziyle dolduruldu
</commit_message>
<xml_diff>
--- a/data/kullanim-defteri.xlsx
+++ b/data/kullanim-defteri.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -740,64 +740,6 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
-        <is>
-          <t>hayir</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>08:40</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>gunluk</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
         <is>
           <t>hayir</t>
         </is>
@@ -877,7 +819,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deftere 'yazan_dagilimi' kolonu: gunluk rapor bolum-bazli uretildiginden tek 'yazan model' yeterli degil — bolum basina model sayaci (bot._LLM_YAZARLAR) ve dagilim kolonu (orn. DeepSeek x5, GLM x3, Nemotron x2, gpt-oss x1). Bugunku gunluk satiri log analizinden gercek dagilimla dolduruldu
</commit_message>
<xml_diff>
--- a/data/kullanim-defteri.xlsx
+++ b/data/kullanim-defteri.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -433,6 +433,7 @@
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,6 +497,11 @@
           <t>rozet</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>yazan_dagilimi</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -558,6 +564,7 @@
           <t>hayir</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -620,6 +627,7 @@
           <t>hayir</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -682,6 +690,7 @@
           <t>hayir</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -742,6 +751,70 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>hayir</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>gunluk</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>karisik (4 model, 11 bolum)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>hayir</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>ZAI/glm-5.3-flash x3, AMD/DeepSeek-V4-Flash x5, NVID/glm-5.3 x2, OR/nemotron x2, YEDEK/gpt-oss-120b x1</t>
         </is>
       </c>
     </row>
@@ -819,7 +892,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Defter: kosu-toplami token kolonlari (kosu_token_in/out) — kabul edilmeyen denemelerin harcamasi dahil GERCEK maliyet gorunur; _llm_call_ic + 3 dogrudan yolun hepsinde _LLM_KOSU_TOKEN birikir. Not: 10/8 derin satirindaki space-bunny metni YAYINLANDI (deneme 5 basarili, kanit: koşu logu) — 'yedek=yazisi cikmaz' degil
</commit_message>
<xml_diff>
--- a/data/kullanim-defteri.xlsx
+++ b/data/kullanim-defteri.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -434,6 +434,8 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,6 +504,16 @@
           <t>yazan_dagilimi</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>kosu_token_in</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>kosu_token_out</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -565,6 +577,16 @@
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -628,6 +650,16 @@
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -691,6 +723,16 @@
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -754,6 +796,16 @@
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -815,6 +867,16 @@
       <c r="M6" t="inlineStr">
         <is>
           <t>ZAI/glm-5.3-flash x3, AMD/DeepSeek-V4-Flash x5, NVID/glm-5.3 x2, OR/nemotron x2, YEDEK/gpt-oss-120b x1</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>